<commit_message>
Use PDF template overlay for integrity pledge
</commit_message>
<xml_diff>
--- a/templates/승락서,지급각서,하자각서.xlsx
+++ b/templates/승락서,지급각서,하자각서.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\진광진광\Desktop\소액공사 자료\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\kist-report-app\project\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA18843-B269-471E-8703-4F85AFC41BCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B7E8504-9C46-4673-8D6A-B2F2097E211B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{AF106CF9-26C5-4562-8BE5-8A8344A1C819}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{AF106CF9-26C5-4562-8BE5-8A8344A1C819}"/>
   </bookViews>
   <sheets>
     <sheet name="★자료입력" sheetId="1" state="hidden" r:id="rId1"/>
@@ -38,9 +38,10 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -1349,6 +1350,51 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="182" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="183" fontId="8" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1376,15 +1422,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="183" fontId="8" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="181" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1410,42 +1447,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="182" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1531,7 +1532,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="승락서(7.5%)"/>
@@ -1573,9 +1574,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1613,7 +1614,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1719,7 +1720,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1861,7 +1862,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3616,45 +3617,45 @@
       <c r="P1" s="17"/>
     </row>
     <row r="2" spans="1:62" s="52" customFormat="1" ht="63.75" customHeight="1">
-      <c r="A2" s="164" t="s">
+      <c r="A2" s="143" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="165"/>
-      <c r="C2" s="165"/>
-      <c r="D2" s="165"/>
-      <c r="E2" s="165"/>
-      <c r="F2" s="165"/>
-      <c r="G2" s="165"/>
-      <c r="H2" s="165"/>
-      <c r="I2" s="165"/>
-      <c r="J2" s="165"/>
-      <c r="K2" s="165"/>
-      <c r="L2" s="165"/>
-      <c r="M2" s="165"/>
-      <c r="N2" s="165"/>
-      <c r="O2" s="165"/>
-      <c r="P2" s="166"/>
+      <c r="B2" s="144"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="144"/>
+      <c r="J2" s="144"/>
+      <c r="K2" s="144"/>
+      <c r="L2" s="144"/>
+      <c r="M2" s="144"/>
+      <c r="N2" s="144"/>
+      <c r="O2" s="144"/>
+      <c r="P2" s="145"/>
     </row>
     <row r="3" spans="1:62" s="19" customFormat="1" ht="29.25" customHeight="1">
       <c r="A3" s="93" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="167" t="str">
+      <c r="B3" s="146" t="str">
         <f>★자료입력!J2</f>
         <v>수소에너지소재연구단(0184호) 청정수소 분리판 기술 개발실 구축(설비)</v>
       </c>
-      <c r="C3" s="168"/>
-      <c r="D3" s="168"/>
-      <c r="E3" s="168"/>
-      <c r="F3" s="168"/>
-      <c r="G3" s="168"/>
-      <c r="H3" s="168"/>
-      <c r="I3" s="168"/>
-      <c r="J3" s="168"/>
-      <c r="K3" s="168"/>
-      <c r="L3" s="168"/>
-      <c r="M3" s="168"/>
-      <c r="N3" s="168"/>
+      <c r="C3" s="147"/>
+      <c r="D3" s="147"/>
+      <c r="E3" s="147"/>
+      <c r="F3" s="147"/>
+      <c r="G3" s="147"/>
+      <c r="H3" s="147"/>
+      <c r="I3" s="147"/>
+      <c r="J3" s="147"/>
+      <c r="K3" s="147"/>
+      <c r="L3" s="147"/>
+      <c r="M3" s="147"/>
+      <c r="N3" s="147"/>
       <c r="O3" s="94" t="s">
         <v>76</v>
       </c>
@@ -3681,26 +3682,26 @@
       <c r="A4" s="93" t="s">
         <v>78</v>
       </c>
-      <c r="B4" s="169" t="str">
+      <c r="B4" s="148" t="str">
         <f>LEFT(★자료입력!I2,4)&amp;"년"&amp;MID(★자료입력!I2,6,2)&amp;"월"&amp;MID(★자료입력!I2,9,2)&amp;"일"</f>
         <v>2025년09월26일</v>
       </c>
-      <c r="C4" s="170"/>
-      <c r="D4" s="170"/>
-      <c r="E4" s="170"/>
-      <c r="F4" s="170"/>
+      <c r="C4" s="149"/>
+      <c r="D4" s="149"/>
+      <c r="E4" s="149"/>
+      <c r="F4" s="149"/>
       <c r="G4" s="58" t="s">
         <v>79</v>
       </c>
       <c r="H4" s="58"/>
-      <c r="I4" s="171" t="str">
+      <c r="I4" s="150" t="str">
         <f>MID(★자료입력!I2,12,4)&amp;"년"&amp;MID(★자료입력!I2,17,2)&amp;"월"&amp;RIGHT(★자료입력!I2,2)&amp;"일"</f>
         <v>2025년10월17일</v>
       </c>
-      <c r="J4" s="171"/>
-      <c r="K4" s="171"/>
-      <c r="L4" s="171"/>
-      <c r="M4" s="171"/>
+      <c r="J4" s="150"/>
+      <c r="K4" s="150"/>
+      <c r="L4" s="150"/>
+      <c r="M4" s="150"/>
       <c r="N4" s="99" t="s">
         <v>80</v>
       </c>
@@ -3715,7 +3716,7 @@
       <c r="AE4" s="29"/>
     </row>
     <row r="5" spans="1:62" ht="23.25" customHeight="1">
-      <c r="A5" s="152" t="s">
+      <c r="A5" s="151" t="s">
         <v>82</v>
       </c>
       <c r="B5" s="101" t="str">
@@ -3735,28 +3736,28 @@
       </c>
       <c r="L5" s="76"/>
       <c r="M5" s="103"/>
-      <c r="N5" s="172">
+      <c r="N5" s="153">
         <f>C6/1.1</f>
         <v>2536363.6363636362</v>
       </c>
-      <c r="O5" s="172"/>
-      <c r="P5" s="173"/>
+      <c r="O5" s="153"/>
+      <c r="P5" s="154"/>
       <c r="AA5" s="62" t="s">
         <v>84</v>
       </c>
       <c r="AB5" s="19"/>
     </row>
     <row r="6" spans="1:62" ht="23.25" customHeight="1">
-      <c r="A6" s="153"/>
+      <c r="A6" s="152"/>
       <c r="B6" s="104"/>
-      <c r="C6" s="154">
+      <c r="C6" s="155">
         <f>★자료입력!L2</f>
         <v>2790000</v>
       </c>
-      <c r="D6" s="154"/>
-      <c r="E6" s="154"/>
-      <c r="F6" s="154"/>
-      <c r="G6" s="154"/>
+      <c r="D6" s="155"/>
+      <c r="E6" s="155"/>
+      <c r="F6" s="155"/>
+      <c r="G6" s="155"/>
       <c r="H6" s="105" t="s">
         <v>68</v>
       </c>
@@ -3767,12 +3768,12 @@
       </c>
       <c r="L6" s="106"/>
       <c r="M6" s="106"/>
-      <c r="N6" s="174">
+      <c r="N6" s="156">
         <f>N5*0.1</f>
         <v>253636.36363636365</v>
       </c>
-      <c r="O6" s="174"/>
-      <c r="P6" s="175"/>
+      <c r="O6" s="156"/>
+      <c r="P6" s="157"/>
       <c r="AA6" s="62" t="s">
         <v>86</v>
       </c>
@@ -3780,7 +3781,7 @@
       <c r="AC6" s="107"/>
     </row>
     <row r="7" spans="1:62" ht="22.5" customHeight="1">
-      <c r="A7" s="152" t="s">
+      <c r="A7" s="151" t="s">
         <v>87</v>
       </c>
       <c r="B7" s="75" t="str">
@@ -3809,18 +3810,18 @@
       <c r="AB7" s="19"/>
     </row>
     <row r="8" spans="1:62" s="19" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A8" s="153"/>
+      <c r="A8" s="152"/>
       <c r="B8" s="104" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="154">
+      <c r="C8" s="155">
         <f>C6*0.15</f>
         <v>418500</v>
       </c>
-      <c r="D8" s="154"/>
-      <c r="E8" s="154"/>
-      <c r="F8" s="154"/>
-      <c r="G8" s="154"/>
+      <c r="D8" s="155"/>
+      <c r="E8" s="155"/>
+      <c r="F8" s="155"/>
+      <c r="G8" s="155"/>
       <c r="H8" s="110" t="s">
         <v>68</v>
       </c>
@@ -3840,53 +3841,53 @@
       <c r="A9" s="93" t="s">
         <v>91</v>
       </c>
-      <c r="B9" s="155" t="s">
+      <c r="B9" s="167" t="s">
         <v>92</v>
       </c>
-      <c r="C9" s="156"/>
-      <c r="D9" s="156"/>
-      <c r="E9" s="156"/>
-      <c r="F9" s="156"/>
-      <c r="G9" s="157"/>
-      <c r="H9" s="158" t="s">
+      <c r="C9" s="168"/>
+      <c r="D9" s="168"/>
+      <c r="E9" s="168"/>
+      <c r="F9" s="168"/>
+      <c r="G9" s="169"/>
+      <c r="H9" s="170" t="s">
         <v>93</v>
       </c>
-      <c r="I9" s="159"/>
-      <c r="J9" s="159"/>
-      <c r="K9" s="159"/>
-      <c r="L9" s="160"/>
-      <c r="M9" s="161" t="s">
+      <c r="I9" s="171"/>
+      <c r="J9" s="171"/>
+      <c r="K9" s="171"/>
+      <c r="L9" s="172"/>
+      <c r="M9" s="173" t="s">
         <v>94</v>
       </c>
-      <c r="N9" s="162"/>
-      <c r="O9" s="162"/>
-      <c r="P9" s="163"/>
+      <c r="N9" s="174"/>
+      <c r="O9" s="174"/>
+      <c r="P9" s="175"/>
     </row>
     <row r="10" spans="1:62" s="19" customFormat="1" ht="30" customHeight="1">
       <c r="A10" s="93" t="s">
         <v>95</v>
       </c>
-      <c r="B10" s="161" t="s">
+      <c r="B10" s="173" t="s">
         <v>96</v>
       </c>
-      <c r="C10" s="162"/>
-      <c r="D10" s="162"/>
-      <c r="E10" s="162"/>
-      <c r="F10" s="162"/>
-      <c r="G10" s="163"/>
-      <c r="H10" s="158" t="s">
+      <c r="C10" s="174"/>
+      <c r="D10" s="174"/>
+      <c r="E10" s="174"/>
+      <c r="F10" s="174"/>
+      <c r="G10" s="175"/>
+      <c r="H10" s="170" t="s">
         <v>97</v>
       </c>
-      <c r="I10" s="159"/>
-      <c r="J10" s="159"/>
-      <c r="K10" s="159"/>
-      <c r="L10" s="160"/>
-      <c r="M10" s="161" t="s">
+      <c r="I10" s="171"/>
+      <c r="J10" s="171"/>
+      <c r="K10" s="171"/>
+      <c r="L10" s="172"/>
+      <c r="M10" s="173" t="s">
         <v>98</v>
       </c>
-      <c r="N10" s="162"/>
-      <c r="O10" s="162"/>
-      <c r="P10" s="163"/>
+      <c r="N10" s="174"/>
+      <c r="O10" s="174"/>
+      <c r="P10" s="175"/>
       <c r="AA10" s="98" t="s">
         <v>99</v>
       </c>
@@ -3949,24 +3950,24 @@
       <c r="BJ11" s="19"/>
     </row>
     <row r="12" spans="1:62" ht="23.25" customHeight="1">
-      <c r="A12" s="143" t="s">
+      <c r="A12" s="158" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="144"/>
-      <c r="C12" s="144"/>
-      <c r="D12" s="144"/>
-      <c r="E12" s="144"/>
-      <c r="F12" s="144"/>
-      <c r="G12" s="144"/>
-      <c r="H12" s="144"/>
-      <c r="I12" s="144"/>
-      <c r="J12" s="144"/>
-      <c r="K12" s="144"/>
-      <c r="L12" s="144"/>
-      <c r="M12" s="144"/>
-      <c r="N12" s="144"/>
-      <c r="O12" s="144"/>
-      <c r="P12" s="145"/>
+      <c r="B12" s="159"/>
+      <c r="C12" s="159"/>
+      <c r="D12" s="159"/>
+      <c r="E12" s="159"/>
+      <c r="F12" s="159"/>
+      <c r="G12" s="159"/>
+      <c r="H12" s="159"/>
+      <c r="I12" s="159"/>
+      <c r="J12" s="159"/>
+      <c r="K12" s="159"/>
+      <c r="L12" s="159"/>
+      <c r="M12" s="159"/>
+      <c r="N12" s="159"/>
+      <c r="O12" s="159"/>
+      <c r="P12" s="160"/>
       <c r="AA12" s="19"/>
       <c r="AB12" s="19"/>
       <c r="AC12" s="19" t="s">
@@ -4004,64 +4005,64 @@
       <c r="BG12" s="19"/>
     </row>
     <row r="13" spans="1:62" ht="23.25" customHeight="1">
-      <c r="A13" s="143"/>
-      <c r="B13" s="144"/>
-      <c r="C13" s="144"/>
-      <c r="D13" s="144"/>
-      <c r="E13" s="144"/>
-      <c r="F13" s="144"/>
-      <c r="G13" s="144"/>
-      <c r="H13" s="144"/>
-      <c r="I13" s="144"/>
-      <c r="J13" s="144"/>
-      <c r="K13" s="144"/>
-      <c r="L13" s="144"/>
-      <c r="M13" s="144"/>
-      <c r="N13" s="144"/>
-      <c r="O13" s="144"/>
-      <c r="P13" s="145"/>
+      <c r="A13" s="158"/>
+      <c r="B13" s="159"/>
+      <c r="C13" s="159"/>
+      <c r="D13" s="159"/>
+      <c r="E13" s="159"/>
+      <c r="F13" s="159"/>
+      <c r="G13" s="159"/>
+      <c r="H13" s="159"/>
+      <c r="I13" s="159"/>
+      <c r="J13" s="159"/>
+      <c r="K13" s="159"/>
+      <c r="L13" s="159"/>
+      <c r="M13" s="159"/>
+      <c r="N13" s="159"/>
+      <c r="O13" s="159"/>
+      <c r="P13" s="160"/>
       <c r="AA13" s="19" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:62" ht="23.25" customHeight="1">
-      <c r="A14" s="143"/>
-      <c r="B14" s="144"/>
-      <c r="C14" s="144"/>
-      <c r="D14" s="144"/>
-      <c r="E14" s="144"/>
-      <c r="F14" s="144"/>
-      <c r="G14" s="144"/>
-      <c r="H14" s="144"/>
-      <c r="I14" s="144"/>
-      <c r="J14" s="144"/>
-      <c r="K14" s="144"/>
-      <c r="L14" s="144"/>
-      <c r="M14" s="144"/>
-      <c r="N14" s="144"/>
-      <c r="O14" s="144"/>
-      <c r="P14" s="145"/>
+      <c r="A14" s="158"/>
+      <c r="B14" s="159"/>
+      <c r="C14" s="159"/>
+      <c r="D14" s="159"/>
+      <c r="E14" s="159"/>
+      <c r="F14" s="159"/>
+      <c r="G14" s="159"/>
+      <c r="H14" s="159"/>
+      <c r="I14" s="159"/>
+      <c r="J14" s="159"/>
+      <c r="K14" s="159"/>
+      <c r="L14" s="159"/>
+      <c r="M14" s="159"/>
+      <c r="N14" s="159"/>
+      <c r="O14" s="159"/>
+      <c r="P14" s="160"/>
       <c r="AA14" s="19" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:62" ht="23.25" customHeight="1">
-      <c r="A15" s="143"/>
-      <c r="B15" s="144"/>
-      <c r="C15" s="144"/>
-      <c r="D15" s="144"/>
-      <c r="E15" s="144"/>
-      <c r="F15" s="144"/>
-      <c r="G15" s="144"/>
-      <c r="H15" s="144"/>
-      <c r="I15" s="144"/>
-      <c r="J15" s="144"/>
-      <c r="K15" s="144"/>
-      <c r="L15" s="144"/>
-      <c r="M15" s="144"/>
-      <c r="N15" s="144"/>
-      <c r="O15" s="144"/>
-      <c r="P15" s="145"/>
+      <c r="A15" s="158"/>
+      <c r="B15" s="159"/>
+      <c r="C15" s="159"/>
+      <c r="D15" s="159"/>
+      <c r="E15" s="159"/>
+      <c r="F15" s="159"/>
+      <c r="G15" s="159"/>
+      <c r="H15" s="159"/>
+      <c r="I15" s="159"/>
+      <c r="J15" s="159"/>
+      <c r="K15" s="159"/>
+      <c r="L15" s="159"/>
+      <c r="M15" s="159"/>
+      <c r="N15" s="159"/>
+      <c r="O15" s="159"/>
+      <c r="P15" s="160"/>
       <c r="AA15" s="19" t="s">
         <v>36</v>
       </c>
@@ -4243,25 +4244,25 @@
       <c r="AK22" s="134"/>
     </row>
     <row r="23" spans="1:62" s="19" customFormat="1" ht="18" customHeight="1">
-      <c r="A23" s="146" t="str">
+      <c r="A23" s="161" t="str">
         <f>LEFT(★자료입력!H2,4)&amp;"년"&amp;MID(★자료입력!H2,6,2)&amp;"월"&amp;MID(★자료입력!H2,9,2)&amp;"일"</f>
         <v>2025년09월26일</v>
       </c>
-      <c r="B23" s="147"/>
-      <c r="C23" s="147"/>
-      <c r="D23" s="147"/>
-      <c r="E23" s="147"/>
-      <c r="F23" s="147"/>
-      <c r="G23" s="147"/>
-      <c r="H23" s="147"/>
-      <c r="I23" s="147"/>
-      <c r="J23" s="147"/>
-      <c r="K23" s="147"/>
-      <c r="L23" s="147"/>
-      <c r="M23" s="147"/>
-      <c r="N23" s="147"/>
-      <c r="O23" s="147"/>
-      <c r="P23" s="148"/>
+      <c r="B23" s="162"/>
+      <c r="C23" s="162"/>
+      <c r="D23" s="162"/>
+      <c r="E23" s="162"/>
+      <c r="F23" s="162"/>
+      <c r="G23" s="162"/>
+      <c r="H23" s="162"/>
+      <c r="I23" s="162"/>
+      <c r="J23" s="162"/>
+      <c r="K23" s="162"/>
+      <c r="L23" s="162"/>
+      <c r="M23" s="162"/>
+      <c r="N23" s="162"/>
+      <c r="O23" s="162"/>
+      <c r="P23" s="163"/>
       <c r="AA23" s="62" t="s">
         <v>58</v>
       </c>
@@ -4567,24 +4568,24 @@
       </c>
     </row>
     <row r="34" spans="1:27" ht="26.25">
-      <c r="A34" s="149" t="s">
+      <c r="A34" s="164" t="s">
         <v>118</v>
       </c>
-      <c r="B34" s="150"/>
-      <c r="C34" s="150"/>
-      <c r="D34" s="150"/>
-      <c r="E34" s="150"/>
-      <c r="F34" s="150"/>
-      <c r="G34" s="150"/>
-      <c r="H34" s="150"/>
-      <c r="I34" s="150"/>
-      <c r="J34" s="150"/>
-      <c r="K34" s="150"/>
-      <c r="L34" s="150"/>
-      <c r="M34" s="150"/>
-      <c r="N34" s="150"/>
-      <c r="O34" s="150"/>
-      <c r="P34" s="151"/>
+      <c r="B34" s="165"/>
+      <c r="C34" s="165"/>
+      <c r="D34" s="165"/>
+      <c r="E34" s="165"/>
+      <c r="F34" s="165"/>
+      <c r="G34" s="165"/>
+      <c r="H34" s="165"/>
+      <c r="I34" s="165"/>
+      <c r="J34" s="165"/>
+      <c r="K34" s="165"/>
+      <c r="L34" s="165"/>
+      <c r="M34" s="165"/>
+      <c r="N34" s="165"/>
+      <c r="O34" s="165"/>
+      <c r="P34" s="166"/>
     </row>
     <row r="35" spans="1:27" ht="16.5">
       <c r="A35" s="46"/>
@@ -4627,14 +4628,6 @@
     <row r="39" spans="1:27" ht="3.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="B3:N3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="I4:M4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="N5:P5"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="N6:P6"/>
     <mergeCell ref="A12:P15"/>
     <mergeCell ref="A23:P23"/>
     <mergeCell ref="A34:P34"/>
@@ -4646,6 +4639,14 @@
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="H10:L10"/>
     <mergeCell ref="M10:P10"/>
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="B3:N3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="I4:M4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="N5:P5"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="N6:P6"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -5703,17 +5704,17 @@
     </row>
     <row r="34" spans="1:9" ht="26.25">
       <c r="A34" s="17"/>
-      <c r="B34" s="149" t="str">
+      <c r="B34" s="164" t="str">
         <f>승락서!A34</f>
         <v>한국과학기술연구원  원장  귀하</v>
       </c>
-      <c r="C34" s="150"/>
-      <c r="D34" s="150"/>
-      <c r="E34" s="150"/>
-      <c r="F34" s="150"/>
-      <c r="G34" s="150"/>
-      <c r="H34" s="150"/>
-      <c r="I34" s="151"/>
+      <c r="C34" s="165"/>
+      <c r="D34" s="165"/>
+      <c r="E34" s="165"/>
+      <c r="F34" s="165"/>
+      <c r="G34" s="165"/>
+      <c r="H34" s="165"/>
+      <c r="I34" s="166"/>
     </row>
     <row r="35" spans="1:9" ht="26.25" customHeight="1">
       <c r="B35" s="48"/>
@@ -6794,8 +6795,8 @@
         <v>43</v>
       </c>
       <c r="B26" s="17" t="str">
-        <f>승락서!D31&amp;"     (인)"</f>
-        <v>김강수     (인)     (인)</v>
+        <f>승락서!D31</f>
+        <v>김강수     (인)</v>
       </c>
       <c r="C26" s="17"/>
       <c r="E26" s="17"/>
@@ -6842,18 +6843,18 @@
       <c r="J29" s="47"/>
     </row>
     <row r="30" spans="1:12" ht="26.25">
-      <c r="A30" s="149" t="s">
+      <c r="A30" s="164" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="150"/>
-      <c r="C30" s="150"/>
-      <c r="D30" s="150"/>
-      <c r="E30" s="150"/>
-      <c r="F30" s="150"/>
-      <c r="G30" s="150"/>
-      <c r="H30" s="150"/>
-      <c r="I30" s="150"/>
-      <c r="J30" s="151"/>
+      <c r="B30" s="165"/>
+      <c r="C30" s="165"/>
+      <c r="D30" s="165"/>
+      <c r="E30" s="165"/>
+      <c r="F30" s="165"/>
+      <c r="G30" s="165"/>
+      <c r="H30" s="165"/>
+      <c r="I30" s="165"/>
+      <c r="J30" s="166"/>
     </row>
     <row r="31" spans="1:12" ht="16.5">
       <c r="A31" s="46"/>

</xml_diff>